<commit_message>
Kahve sohbeti farki yuvarlandi
</commit_message>
<xml_diff>
--- a/bolge-kpi-platformu.xlsx
+++ b/bolge-kpi-platformu.xlsx
@@ -1145,7 +1145,7 @@
                   <c:v>78</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>62</c:v>
+                  <c:v>66</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1153,11 +1153,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="45196273"/>
-        <c:axId val="5186709"/>
+        <c:axId val="11043188"/>
+        <c:axId val="29703506"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="45196273"/>
+        <c:axId val="11043188"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1189,7 +1189,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5186709"/>
+        <c:crossAx val="29703506"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1197,7 +1197,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5186709"/>
+        <c:axId val="29703506"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -1241,7 +1241,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45196273"/>
+        <c:crossAx val="11043188"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4953,8 +4953,8 @@
         <v>0.125</v>
       </c>
       <c r="S5" s="17" t="n">
-        <f aca="false">IFERROR(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A5,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A5,Kahve_Sohbeti!$A:$A,0))*0.2*2,"")</f>
-        <v>-2.4</v>
+        <f aca="false">IFERROR(ROUND(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A5,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A5,Kahve_Sohbeti!$A:$A,0))*0.2*2,0),"")</f>
+        <v>-2</v>
       </c>
       <c r="T5" s="18" t="n">
         <f aca="false">IFERROR(INDEX(Sikayet!$E:$E,MATCH($B$1&amp;"|"&amp;$A5,Sikayet!$A:$A,0))/INDEX(Sikayet!$D:$D,MATCH($B$1&amp;"|"&amp;$A5,Sikayet!$A:$A,0))*1000,"")</f>
@@ -5057,8 +5057,8 @@
         <v>0</v>
       </c>
       <c r="S6" s="17" t="n">
-        <f aca="false">IFERROR(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A6,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A6,Kahve_Sohbeti!$A:$A,0))*0.2*2,"")</f>
-        <v>2.6</v>
+        <f aca="false">IFERROR(ROUND(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A6,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A6,Kahve_Sohbeti!$A:$A,0))*0.2*2,0),"")</f>
+        <v>3</v>
       </c>
       <c r="T6" s="18" t="n">
         <f aca="false">IFERROR(INDEX(Sikayet!$E:$E,MATCH($B$1&amp;"|"&amp;$A6,Sikayet!$A:$A,0))/INDEX(Sikayet!$D:$D,MATCH($B$1&amp;"|"&amp;$A6,Sikayet!$A:$A,0))*1000,"")</f>
@@ -5161,8 +5161,8 @@
         <v>0.111111111111111</v>
       </c>
       <c r="S7" s="17" t="n">
-        <f aca="false">IFERROR(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A7,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A7,Kahve_Sohbeti!$A:$A,0))*0.2*2,"")</f>
-        <v>3.4</v>
+        <f aca="false">IFERROR(ROUND(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A7,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A7,Kahve_Sohbeti!$A:$A,0))*0.2*2,0),"")</f>
+        <v>3</v>
       </c>
       <c r="T7" s="18" t="n">
         <f aca="false">IFERROR(INDEX(Sikayet!$E:$E,MATCH($B$1&amp;"|"&amp;$A7,Sikayet!$A:$A,0))/INDEX(Sikayet!$D:$D,MATCH($B$1&amp;"|"&amp;$A7,Sikayet!$A:$A,0))*1000,"")</f>
@@ -5265,8 +5265,8 @@
         <v>0.210526315789474</v>
       </c>
       <c r="S8" s="17" t="n">
-        <f aca="false">IFERROR(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A8,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A8,Kahve_Sohbeti!$A:$A,0))*0.2*2,"")</f>
-        <v>3.4</v>
+        <f aca="false">IFERROR(ROUND(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A8,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A8,Kahve_Sohbeti!$A:$A,0))*0.2*2,0),"")</f>
+        <v>3</v>
       </c>
       <c r="T8" s="18" t="n">
         <f aca="false">IFERROR(INDEX(Sikayet!$E:$E,MATCH($B$1&amp;"|"&amp;$A8,Sikayet!$A:$A,0))/INDEX(Sikayet!$D:$D,MATCH($B$1&amp;"|"&amp;$A8,Sikayet!$A:$A,0))*1000,"")</f>
@@ -5369,8 +5369,8 @@
         <v>0</v>
       </c>
       <c r="S9" s="17" t="n">
-        <f aca="false">IFERROR(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A9,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A9,Kahve_Sohbeti!$A:$A,0))*0.2*2,"")</f>
-        <v>-1.2</v>
+        <f aca="false">IFERROR(ROUND(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A9,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A9,Kahve_Sohbeti!$A:$A,0))*0.2*2,0),"")</f>
+        <v>-1</v>
       </c>
       <c r="T9" s="18" t="n">
         <f aca="false">IFERROR(INDEX(Sikayet!$E:$E,MATCH($B$1&amp;"|"&amp;$A9,Sikayet!$A:$A,0))/INDEX(Sikayet!$D:$D,MATCH($B$1&amp;"|"&amp;$A9,Sikayet!$A:$A,0))*1000,"")</f>
@@ -5473,8 +5473,8 @@
         <v>0.166666666666667</v>
       </c>
       <c r="S10" s="17" t="n">
-        <f aca="false">IFERROR(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A10,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A10,Kahve_Sohbeti!$A:$A,0))*0.2*2,"")</f>
-        <v>0.199999999999999</v>
+        <f aca="false">IFERROR(ROUND(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A10,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A10,Kahve_Sohbeti!$A:$A,0))*0.2*2,0),"")</f>
+        <v>0</v>
       </c>
       <c r="T10" s="18" t="n">
         <f aca="false">IFERROR(INDEX(Sikayet!$E:$E,MATCH($B$1&amp;"|"&amp;$A10,Sikayet!$A:$A,0))/INDEX(Sikayet!$D:$D,MATCH($B$1&amp;"|"&amp;$A10,Sikayet!$A:$A,0))*1000,"")</f>
@@ -5577,7 +5577,7 @@
         <v>0.5</v>
       </c>
       <c r="S11" s="17" t="n">
-        <f aca="false">IFERROR(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A11,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A11,Kahve_Sohbeti!$A:$A,0))*0.2*2,"")</f>
+        <f aca="false">IFERROR(ROUND(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A11,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A11,Kahve_Sohbeti!$A:$A,0))*0.2*2,0),"")</f>
         <v>2</v>
       </c>
       <c r="T11" s="18" t="n">
@@ -5681,8 +5681,8 @@
         <v>0.363636363636364</v>
       </c>
       <c r="S12" s="17" t="n">
-        <f aca="false">IFERROR(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A12,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A12,Kahve_Sohbeti!$A:$A,0))*0.2*2,"")</f>
-        <v>-0.4</v>
+        <f aca="false">IFERROR(ROUND(INDEX(Kahve_Sohbeti!$E:$E,MATCH($B$1&amp;"|"&amp;$A12,Kahve_Sohbeti!$A:$A,0))-INDEX(Kahve_Sohbeti!$D:$D,MATCH($B$1&amp;"|"&amp;$A12,Kahve_Sohbeti!$A:$A,0))*0.2*2,0),"")</f>
+        <v>-0</v>
       </c>
       <c r="T12" s="18" t="n">
         <f aca="false">IFERROR(INDEX(Sikayet!$E:$E,MATCH($B$1&amp;"|"&amp;$A12,Sikayet!$A:$A,0))/INDEX(Sikayet!$D:$D,MATCH($B$1&amp;"|"&amp;$A12,Sikayet!$A:$A,0))*1000,"")</f>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="X12" s="19" t="n">
         <f aca="false">INDEX(Performans_Puani!$S:$S,ROW())</f>
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="Y12" s="20" t="n">
         <f aca="false">IFERROR(RANK(X12,$X$5:$X$12),"")</f>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="S13" s="28" t="n">
         <f aca="false">SUM(S5:S12)</f>
-        <v>7.6</v>
+        <v>8</v>
       </c>
       <c r="T13" s="29" t="n">
         <f aca="false">IFERROR(AVERAGE(T5:T12),"")</f>
@@ -5804,7 +5804,7 @@
       </c>
       <c r="X13" s="30" t="n">
         <f aca="false">IFERROR(AVERAGE(X5:X12),"")</f>
-        <v>62.375</v>
+        <v>62.875</v>
       </c>
       <c r="Y13" s="22"/>
       <c r="Z13" s="22"/>
@@ -6696,7 +6696,7 @@
       </c>
       <c r="M12" s="33" t="n">
         <f aca="false">IF(Genel_Tablo!S12="","",IF(IF(Hedefler!$D$15="≥",Genel_Tablo!S12&gt;=Hedefler!$E$15,Genel_Tablo!S12&lt;=Hedefler!$E$15),Hedefler!$F$15,0))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N12" s="33" t="n">
         <f aca="false">IF(Genel_Tablo!T12="","",IF(IF(Hedefler!$D$16="≥",Genel_Tablo!T12&gt;=Hedefler!$E$16,Genel_Tablo!T12&lt;=Hedefler!$E$16),Hedefler!$F$16,0))</f>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="S12" s="34" t="n">
         <f aca="false">SUM(B12:Q12)</f>
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>